<commit_message>
Bulk commit upload: advancing tutorials.
</commit_message>
<xml_diff>
--- a/docs/source/tutorials/production_planning/materials/model/sets.xlsx
+++ b/docs/source/tutorials/production_planning/materials/model/sets.xlsx
@@ -1,72 +1,64 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\cvxlab\docs\source\tutorials\tutorial_simple\model\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365.sharepoint.com/sites/DENG-SESAM/Documenti condivisi/c-Research/b-Models/CVXlab/tutorials/tutorial_website/model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{711C8911-29A3-464B-B235-A72F53430F54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="11_C95A2D3FD0E4F6B28A5978D88444968BA57FA744" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BBA3F538-7AD9-490E-B954-A8909CD56ADD}"/>
   <bookViews>
-    <workbookView xWindow="5440" yWindow="2360" windowWidth="23460" windowHeight="15450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5240" yWindow="2440" windowWidth="31320" windowHeight="17130" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="_set_RESOURCES" sheetId="1" r:id="rId1"/>
-    <sheet name="_set_PRODUCTS" sheetId="2" r:id="rId2"/>
-    <sheet name="_set_PRODUCT_DATA" sheetId="3" r:id="rId3"/>
+    <sheet name="_set_PRODUCTS" sheetId="1" r:id="rId1"/>
+    <sheet name="_set_ATTRIBUTES" sheetId="2" r:id="rId2"/>
+    <sheet name="_set_SCENARIOS_ENERGY" sheetId="3" r:id="rId3"/>
+    <sheet name="_set_SCENARIOS_MATERIAL" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
-  <si>
-    <t>resources_Name</t>
-  </si>
-  <si>
-    <t>products_Name</t>
-  </si>
-  <si>
-    <t>product_data_Name</t>
-  </si>
-  <si>
-    <t>product_data_category</t>
-  </si>
-  <si>
-    <t>low energy</t>
-  </si>
-  <si>
-    <t>avg energy</t>
-  </si>
-  <si>
-    <t>high energy</t>
-  </si>
-  <si>
-    <t>product 1</t>
-  </si>
-  <si>
-    <t>product 2</t>
-  </si>
-  <si>
-    <t>unit energy use, initial</t>
-  </si>
-  <si>
-    <t>energy_use_0</t>
-  </si>
-  <si>
-    <t>unit profit</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="12">
+  <si>
+    <t>Products_Name</t>
+  </si>
+  <si>
+    <t>Attributes_Name</t>
+  </si>
+  <si>
+    <t>Attributes_type</t>
+  </si>
+  <si>
+    <t>Scenarios_energy_Name</t>
+  </si>
+  <si>
+    <t>Scenarios_material_Name</t>
+  </si>
+  <si>
+    <t>product_1</t>
+  </si>
+  <si>
+    <t>product_2</t>
+  </si>
+  <si>
+    <t>energy</t>
+  </si>
+  <si>
+    <t>material</t>
   </si>
   <si>
     <t>profit</t>
   </si>
   <si>
-    <t>learning rate</t>
-  </si>
-  <si>
-    <t>learning_rate</t>
+    <t>low</t>
+  </si>
+  <si>
+    <t>high</t>
   </si>
 </sst>
 </file>
@@ -429,8 +421,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22.54296875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -439,16 +434,11 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
         <v>6</v>
       </c>
     </row>
@@ -459,22 +449,71 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="21.54296875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -482,44 +521,349 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:B4"/>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22.90625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>11</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5d44ae6a-e145-4c9d-94e7-ddf9cc58067e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="e67e9a88-35e1-4b39-8da9-a609eb308282" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100241E96938535DD4B921FCDFB54345D30" ma:contentTypeVersion="19" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="7b5477e5183001dfb744417d6d3e1bdb">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5d44ae6a-e145-4c9d-94e7-ddf9cc58067e" xmlns:ns3="e67e9a88-35e1-4b39-8da9-a609eb308282" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="47c71bcc7ce4561c40563d7718896ae0" ns2:_="" ns3:_="">
+    <xsd:import namespace="5d44ae6a-e145-4c9d-94e7-ddf9cc58067e"/>
+    <xsd:import namespace="e67e9a88-35e1-4b39-8da9-a609eb308282"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="5d44ae6a-e145-4c9d-94e7-ddf9cc58067e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="10" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceKeyPoints" ma:index="11" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceAutoTags" ma:index="13" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="17" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="22" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Tag immagine" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="62691f12-1220-44b1-ba48-e77f64da2991" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="24" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="26" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e67e9a88-35e1-4b39-8da9-a609eb308282" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Condiviso con" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Condiviso con dettagli" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="TaxCatchAll" ma:index="23" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{cfe7f1f2-b186-4eae-b9db-3e53485d6587}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e67e9a88-35e1-4b39-8da9-a609eb308282">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo di contenuto"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titolo"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{83117F71-DA80-4899-8EAF-E1FFEB571F60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="5d44ae6a-e145-4c9d-94e7-ddf9cc58067e"/>
+    <ds:schemaRef ds:uri="e67e9a88-35e1-4b39-8da9-a609eb308282"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B0E58CA-8C44-4A7B-B92C-F5AFA70F3216}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C95B7511-0554-4546-AA4C-DE4ABDB35B94}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5d44ae6a-e145-4c9d-94e7-ddf9cc58067e"/>
+    <ds:schemaRef ds:uri="e67e9a88-35e1-4b39-8da9-a609eb308282"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>